<commit_message>
update product with image
</commit_message>
<xml_diff>
--- a/backend/data/raw/products.xlsx
+++ b/backend/data/raw/products.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b8827725017ffd42/Documents/GitHub/GROUP_10_TOPIC_10_SEMANTIC_SEARCH/backend/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TVPC\Documents\tl kì 2\2-Advanced Databases\project\GROUP_10_TOPIC_10_SEMANTIC_SEARCH\backend\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_F25DC773A252ABDACC1048B1C15E65C65BDE58F8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD22DD06-4F1D-42D5-A4F4-3CA104A4FA55}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667693E6-60E9-475C-B20E-C088DDFF364E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="513">
   <si>
     <t xml:space="preserve">category_id </t>
   </si>
@@ -1143,6 +1143,468 @@
   </si>
   <si>
     <t>speaker/speaker_10.jpg</t>
+  </si>
+  <si>
+    <t>Tổng Bí Thư Triều Tiên Kim Jong Un</t>
+  </si>
+  <si>
+    <t>North Korea</t>
+  </si>
+  <si>
+    <t>persident/persident_1.jpg</t>
+  </si>
+  <si>
+    <t>Ukraine</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>Tổng Bí Thư Trung Quốc Tập Cận Bình</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Russia</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>Tổng Thống Mỹ Donald Trump</t>
+  </si>
+  <si>
+    <t>Cựu Tổng Thống Mỹ Joe Biden</t>
+  </si>
+  <si>
+    <t>Cựu Tổng Thống Mỹ Bill Clinton</t>
+  </si>
+  <si>
+    <t>Cựu Tổng Thống Mỹ Barack Obama</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>Tổng Thống Ukraine Volodymyr Zelenskyy</t>
+  </si>
+  <si>
+    <t>Thủ Tướng Nhật Bản Takaichi Sanae</t>
+  </si>
+  <si>
+    <t>Tổng Thống Nga Vladimir Putin</t>
+  </si>
+  <si>
+    <t>Cựu Tổng Thống Hàn Quốc Yoon Suk-yeol</t>
+  </si>
+  <si>
+    <t>Thiết kế: Kiểu dáng bo tròn công nghiệp, đi kèm "mái tóc bay" khí động học độc quyền. Tính năng: Chế độ "Dỗi là bắn" cực nhạy. Tích hợp loa phóng thanh công suất lớn, tự động phát nhạc hành khúc 24/7. Lưu ý: Chỉ vận hành tốt nhất tại thị trường nội địa. Không hỗ trợ đổi trả nếu bạn không hài lòng</t>
+  </si>
+  <si>
+    <t>Thiết kế: Tone màu Xanh Rêu Quân Đội xuyên suốt mọi sự kiện, từ hầm trú ẩn đến thảm đỏ Hollywood. Form dáng "không ngủ", tích hợp quầng thâm mắt chính hãng để tăng độ uy tín.
+Tính năng: * Auto-Call: Tự động kết nối với mọi nguyên thủ quốc gia lúc 3 giờ sáng để hỏi mượn... "đồ chơi" hạng nặng.
+Grammy-Filter: Khả năng xuất hiện trên mọi màn hình lớn tại các lễ trao giải dù không có vé mời. Lưu ý: Sản phẩm cực kỳ tốn kém để bảo trì. Nếu bạn không gửi "linh kiện" định kỳ, máy sẽ tự động gửi thông báo "Hết đạn" lên toàn cầu</t>
+  </si>
+  <si>
+    <t>Thiết kế: Vỏ ngoài bằng polyme siêu cứng, chống chỉ định với các loại "Gió Tây". Kiểu tóc cố định 100% bằng keo xịt chuyên dụng, bất chấp mọi biến động của thị trường chứng khoán Nikkei. Tính năng: Radar "Yasukuni"-Tự động phát tín hiệu gây nhiễu mỗi khi có ai đó nhắc đến từ "Hòa bình" theo kiểu hiện đại. Phụ kiện: Tặng kèm một bộ lọc chặn hoàn toàn các cuộc gọi từ Bắc Kinh và Seoul để đảm bảo máy không bị "treo".
+Lưu ý: Sản phẩm có thể gây "nóng máy" cực độ nếu đặt cạnh các mặt hàng thuộc dòng Liberal. Chỉ dành cho những người thích hoài niệm về thời kỳ "Mặt trời không bao giờ lặn" (phiên bản Tokyo).</t>
+  </si>
+  <si>
+    <t>Thiết kế: Bền bỉ như xe tăng, vững chãi như một quảng trường không bao giờ có biến cố. Bề mặt nhẵn nhụi, đã được quét sạch mọi "vết xước" lịch sử bằng bộ lọc xóa phông siêu cấp. Tính năng: Zero-COVID Sensor-Cảm biến siêu nhạy, tự động khóa chặt mọi cửa sổ nếu phát hiện một con vi khuẩn đi ngang qua. Phụ kiện: Tặng kèm một chú gấu vàng (đã bị gạch chéo và dán nhãn "Cấm lưu hành") và một bản đồ "Đường lưỡi bò" tự vẽ bằng bút xóa. Trạng thái: Hoàn hảo. Không có lỗi, không có lịch sử, và quan trọng nhất là không có gì để xem ở đây cả.</t>
+  </si>
+  <si>
+    <t>Thiết kế: Vỏ ngoài đúc bằng thép lạnh vùng Siberia, chống thấm nước tuyệt đối (phù hợp cho các hoạt động cởi trần cưỡi gấu). Tính năng: Chế độ "Chiến dịch đặc biệt"-Tự động mở rộng "không gian lưu trữ" sang các ổ đĩa lân cận mà không cần sự đồng ý của admin. GPS "Ngược"-Mọi con đường đều dẫn về Moscow, bất kể bạn đang định vị ở đâu. Khả năng "Hoán đổi linh kiện" (Thủ tướng thành Tổng thống và ngược lại) một cách ảo diệu để duy trì tuổi thọ pin lên đến hàng thập kỷ.</t>
+  </si>
+  <si>
+    <t>Thiết kế: Được gia cố bằng lớp giáp chống biểu tình nhưng lại cực kỳ dễ nứt vỡ trước áp lực từ phía Quốc hội. Tính năng: Chế độ "Thiết quân luật nửa đêm"-Tự động kích hoạt khi cảm thấy bị dồn vào đường cùng; có khả năng biến một quốc gia dân chủ thành phim hành động thập niên 80 chỉ trong 2 tiếng. AI "Lắng nghe vợ"-Tích hợp bộ vi xử lý ưu tiên tuyệt đối mọi mệnh lệnh từ "Phu nhân linh kiện", bỏ qua hoàn toàn cảnh báo lỗi từ hệ thống cử dân. Khả năng "tự hủy" nhanh kỷ lục. Vừa nhấn nút Start đã nhảy thẳng sang chế độ Impeachment (Luận tội). Phụ kiện: Tặng kèm một chiếc máy bay trực thăng đổ bộ nóc tòa nhà Quốc hội và một bản diễn văn xin lỗi được soạn sẵn nhưng không ai thèm nghe. Lưu ý: Sản phẩm có nguy cơ bị thu hồi và chuyển vào kho bảo quản (nhà tù) sớm hơn dự kiến. Không hỗ trợ bảo hành trước các cáo buộc phản quốc.</t>
+  </si>
+  <si>
+    <t>Thiết kế: Vỏ ngoài bằng vật liệu cổ điển, đôi khi xuất hiện các vết nứt do thời gian nhưng luôn được đánh bóng bằng một chiếc kính phi công Ray-Ban cực ngầu. Tính năng: * GPS "Lạc lối": Tích hợp bản đồ thế giới nhưng thỉnh thoảng tự động rẽ nhầm hướng khi bước xuống sân khấu hoặc tìm lối ra sau bài phát biểu. Whisper Mode: Chế độ thì thầm vào mic cực kỳ kịch tính, khiến đối phương vừa bối rối vừa phải tự hỏi: "Ông ấy vừa nói gì thế?". Khả năng "Đóng băng" (Freeze) cực kỳ chân thực. Máy có thể đứng yên hoàn hảo trong 30 giây giữa một sự kiện sôi động, tạo cảm giác như mạng đang bị lag.</t>
+  </si>
+  <si>
+    <t>Thiết kế: Bọc lớp vỏ màu cam rực rỡ "Indestructible", mái tóc được khí động học hóa để chịu được sức gió từ cánh quạt trực thăng. Tính năng: * Tariff Shield: Tự động dựng tường lửa thu thuế mọi mặt hàng xung quanh, bất kể là đồng minh hay đối thủ. Social Media Blast: Khả năng xuất bản 100 thông báo "CHƯA TỪNG CÓ" mỗi phút, khiến mọi hệ thống kiểm duyệt đều bị quá tải. Chế độ "Unsinkable" (Không thể chìm). Dù bị va đập bởi tòa án, luận tội hay "vật thể lạ" bay ngang tai, mặt hàng này vẫn tự động đứng dậy, giơ nắm đấm và hô "Fight!". Phụ kiện: Tặng kèm một chiếc mũ đỏ có khả năng tăng 100% chỉ số tự tin và một tài khoản ngân hàng không giới hạn</t>
+  </si>
+  <si>
+    <t>Thiết kế: Vỏ ngoài trơn láng, bọc da cao cấp với khả năng co giãn linh hoạt trước mọi sự truy vấn. Phong cách lãng tử thập niên 90 nhưng lại có sở thích phiêu lưu ở những hòn đảo xa xôi. Tính năng: Island Hopper Mode-Tự động kích hoạt chế độ "không lưu lại lịch trình" khi di chuyển trên các dòng chuyên cơ tư nhân, đặc biệt là dòng "Lolita Express". Cảnh báo: Không nên để mặt hàng này hoạt động một mình trong phòng kín với các "linh kiện" thực tập sinh trẻ tuổi. Rất dễ xảy ra hiện tượng "chập mạch" đạo đức. Sản phẩm có thể gây dị ứng mạnh cho những ai ưa thích sự minh bạch. Tuyệt đối không để gần các khu vực có camera an ninh hoạt động ổn định</t>
+  </si>
+  <si>
+    <t>Thiết kế: Tone màu "Hòa hợp dân tộc" bóng bẩy, phong cách thời trang chuẩn quý ông nghỉ hưu với những bộ suit không tì vết. Đặc biệt tích hợp bộ lọc "Cool-Guy" khiến mọi hành động, dù là ném bom hay đi dạo, đều trông như một cảnh phim điện ảnh. Tính năng: Khả năng đạt giải Nobel Hòa bình theo hình thức "trả góp niềm tin" – nhận giải trước, làm việc (hoặc không) sau. Phụ kiện: Một hợp đồng sản xuất phim triệu đô với Netflix để kể về cuộc đời mình một cách khiêm tốn nhất có thể. Một danh sách nghe nhạc Spotify được dàn dựng công phu để chứng minh rằng "Tôi vẫn rất trẻ trung và hợp thời". Lưu ý: Sản phẩm có tính năng "Nói cực hay nhưng làm thì... từ từ". Rất giỏi trong việc truyền cảm hứng cho bạn tin vào sự thay đổi, trong khi thực tế hệ thống vẫn giữ nguyên cấu hình cũ.</t>
+  </si>
+  <si>
+    <t>F-22 Raptor</t>
+  </si>
+  <si>
+    <t>F-35 Lightning II</t>
+  </si>
+  <si>
+    <t>Su-57 Felon</t>
+  </si>
+  <si>
+    <t>J-20 Mighty Dragon</t>
+  </si>
+  <si>
+    <t>B-2 Spirit</t>
+  </si>
+  <si>
+    <t>"Siêu phẩm đời đầu" nhưng chưa bao giờ lỗi mốt. Đây là mẫu máy bay mà chính phủ Mỹ ích kỷ đến mức cấm xuất khẩu cho bất kỳ ai. Nó tàng hình tốt đến mức radar đối phương thường nhầm nó với một con chim sẻ đang bay ở vận tốc siêu thanh.</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_10.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_01.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_02.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_03.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_04.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_05.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_06.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_09.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_08.jpg</t>
+  </si>
+  <si>
+    <t>stealth aircraft/stealthAircraft_07.jpg</t>
+  </si>
+  <si>
+    <t>Chiếc "iPhone" của giới không quân. Nó đầy rẫy công nghệ và phần mềm phức tạp, đôi khi gặp lỗi cập nhật (bug), nhưng một khi đã chạy mượt thì nó sẽ kết nối mọi thứ trên chiến trường vào màn hình của phi công như chơi game.</t>
+  </si>
+  <si>
+    <t>Một gã lực sĩ cơ bắp từ Nga. Dù khả năng tàng hình còn gây tranh cãi (bị mỉa mai là chỉ tàng hình được một nửa), nhưng về khoản nhào lộn và thực chiến đối đầu trực diện, nó là một đối thủ cực kỳ khó chịu.</t>
+  </si>
+  <si>
+    <t>"Con rồng" khổng lồ với sải cánh dài ngoằng. Nó được thiết kế để bay xa và ám sát các máy bay hậu cần của đối phương. Một sự kết hợp thú vị giữa ý tưởng phương Tây và nhu cầu "phủ sóng" phương Đông.</t>
+  </si>
+  <si>
+    <t>Một chiếc "phi thuyền người ngoài hành tinh" đúng nghĩa. Nó không có đuôi, bay lơ lửng như một bóng ma và có mức giá khiến người ta phải rùng mình hơn cả sức mạnh hủy diệt của nó.</t>
+  </si>
+  <si>
+    <t>B-21 Raider</t>
+  </si>
+  <si>
+    <t>Phiên bản "tối ưu hóa chi phí" của B-2. Nó nhỏ hơn, thông minh hơn và được sinh ra để làm công việc ném bom trở nên... kinh tế hơn trong kỷ nguyên số.</t>
+  </si>
+  <si>
+    <t>J-35 / FC-31</t>
+  </si>
+  <si>
+    <t>Em trai của J-20, trông giống hệt F-35 nhưng được "made in China". Nó được sinh ra để đáp xuống tàu sân bay và chứng minh rằng Trung Quốc có thể sản xuất mọi thứ mà phương Tây có.</t>
+  </si>
+  <si>
+    <t>KF-21 Boramae</t>
+  </si>
+  <si>
+    <t>Một sản phẩm của sự kiên trì. Hàn Quốc muốn tự xây dựng một hệ thống tàng hình riêng để không phải "nhìn sắc mặt" nhà cung cấp ngoại quốc. Ngoại hình rất giống F-22 nhưng mang linh hồn K-Pop hiện đại.</t>
+  </si>
+  <si>
+    <t>KAAN</t>
+  </si>
+  <si>
+    <t>Niềm tự hào của Thổ Nhĩ Kỳ. Đây là lời khẳng định rằng họ có thể tự làm siêu máy bay tàng hình sau khi bị Mỹ "kick" khỏi dự án F-35. Một mặt hàng đầy tham trọng chính trị.</t>
+  </si>
+  <si>
+    <t>F-117 Nighthawk</t>
+  </si>
+  <si>
+    <t>Turkey</t>
+  </si>
+  <si>
+    <t>"Cụ tổ" của ngành tàng hình. Với những đường nét góc cạnh như một viên kim cương đen, dù đã chính thức nghỉ hưu nhưng thỉnh thoảng cụ vẫn xuất hiện trên bầu trời để dạy bảo các hậu bối.</t>
+  </si>
+  <si>
+    <t>Little Boy</t>
+  </si>
+  <si>
+    <t>Loại bom nguyên tử đầu tiên được sử dụng trong chiến tranh (thả xuống Hiroshima). Nó có thiết kế kiểu "súng" đơn giản nhưng hiệu quả kinh khủng, biến một thành phố thành tro bụi chỉ trong tích tắc.</t>
+  </si>
+  <si>
+    <t>Fat Man</t>
+  </si>
+  <si>
+    <t>"Người anh em" to béo hơn thả xuống Nagasaki. Sử dụng lõi Plutonium với cơ chế nổ lõm phức tạp hơn Little Boy. Ngoại hình trông như một quả trứng khổng lồ mang theo lời nguyền diệt vong.</t>
+  </si>
+  <si>
+    <t>Tsar Bomba</t>
+  </si>
+  <si>
+    <t>"Vua của các loại bom". Đây là vũ khí hạt nhân mạnh nhất từng được kích nổ trong lịch sử nhân loại. Sức mạnh của nó khủng khiếp đến mức sóng chấn động đã đi vòng quanh trái đất ba lần.</t>
+  </si>
+  <si>
+    <t>B83</t>
+  </si>
+  <si>
+    <t>B61-12</t>
+  </si>
+  <si>
+    <t>RDS-1</t>
+  </si>
+  <si>
+    <t>Quả bom nguyên tử đầu tiên của Liên Xô, chấm dứt thế độc tôn hạt nhân của Mỹ. Nó có thiết kế khá giống với Fat Man của Mỹ (nhờ một chút "hỗ trợ" từ tình báo).</t>
+  </si>
+  <si>
+    <t>RS-28 Sarmat / Satan 2</t>
+  </si>
+  <si>
+    <t>Không chỉ là một quả bom, đây là một con quái vật mang nhiều đầu đạn hạt nhân. Một tên lửa đơn lẻ có thể mang đủ sức mạnh để xóa sổ một khu vực rộng lớn bằng diện tích nước Pháp.</t>
+  </si>
+  <si>
+    <t>Dongfeng-41 / DF-41</t>
+  </si>
+  <si>
+    <t>Tên lửa hành trình liên lục địa có tầm bắn xa nhất thế giới hiện nay, mang theo nhiều đầu đạn hạt nhân độc lập (MIRV) có khả năng xuyên thủng mọi hệ thống phòng thủ.</t>
+  </si>
+  <si>
+    <t>LGM-30G Minuteman III</t>
+  </si>
+  <si>
+    <t>Xương sống của lực lượng răn đe hạt nhân trên đất liền của Mỹ. Những "lão tướng" này luôn nằm sẵn trong các giếng phóng dưới lòng đất, trực chiến 24/7.</t>
+  </si>
+  <si>
+    <t>Trident II D5</t>
+  </si>
+  <si>
+    <t>Loại tên lửa hạt nhân phóng từ tàu ngầm cực kỳ lợi hại. Vì nằm dưới đại dương nên nó gần như không thể bị phát hiện trước khi phóng, là đòn trả đũa kinh hoàng từ lòng biển.</t>
+  </si>
+  <si>
+    <t>Chuyên gia "đào bới" dành cho những ai thích chơi trốn tìm dưới lòng đất. B83 được thiết kế để đập tan sự tự tin của những chiếc hầm trú ẩn kiên cố nhất. Nó giống như một chiếc búa tạ khổng lồ gõ thẳng vào đầu những kẻ thích xây nhà dưới hầm.</t>
+  </si>
+  <si>
+    <t>Mẫu "Smart-bomb" dành cho thế kỷ 21. Với khả năng điều chỉnh sức công phá, bạn có thể chọn chế độ "vừa đủ để xóa sổ một sân bay" hoặc "thổi bay cả một quân đoàn". Nó nhỏ gọn đến mức có thể nhét vừa khoang bụng của mấy chiếc tiêm kích tàng hình bạn vừa xem ở trên.</t>
+  </si>
+  <si>
+    <t>bomb/bomb_01.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_02.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_03.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_04.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_05.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_06.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_07.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_08.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_09.jpg</t>
+  </si>
+  <si>
+    <t>bomb/bomb_10.jpg</t>
+  </si>
+  <si>
+    <t>AK-47</t>
+  </si>
+  <si>
+    <t>gun/gun_01.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_02.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_03.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_04.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_05.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_06.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_07.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_08.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_09.jpg</t>
+  </si>
+  <si>
+    <t>gun/gun_10.jpg</t>
+  </si>
+  <si>
+    <t>Món đồ không thể thiếu cho những ai ưa thích sự thực dụng. Với cơ chế vận hành đơn giản đến mức khó tin, AK-47 thách thức mọi điều kiện thời tiết từ bão cát sa mạc đến bùn lầy rừng rậm. Đây là biểu tượng của sức mạnh bền bỉ, mua một lần, dùng cả đời.</t>
+  </si>
+  <si>
+    <t>M4A1 Carbine</t>
+  </si>
+  <si>
+    <t>Sự kết hợp hoàn hảo giữa độ chính xác và tính linh hoạt. M4A1 cho phép bạn tùy biến mọi phụ kiện từ kính ngắm laser đến tay cầm hiện đại. Trọng lượng nhẹ, độ giật thấp, đây là lựa chọn hàng đầu cho các chuyên gia yêu cầu sự tinh tế trên chiến trường.</t>
+  </si>
+  <si>
+    <t>Desert Eagle .50 AE</t>
+  </si>
+  <si>
+    <t>Mặt hàng dành riêng cho những người thích phô trương sức mạnh. Với vẻ ngoài mạ chrome bóng bẩy và cỡ đạn khổng lồ, Desert Eagle không chỉ là một khẩu súng, nó là một tuyên ngôn về quyền lực. Lưu ý: Cần một đôi tay thép để chế ngự con quái vật này.</t>
+  </si>
+  <si>
+    <t>Glock 17</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Một siêu phẩm làm từ polymer cao cấp với thiết kế tối giản. Glock 17 loại bỏ mọi rườm rà để tập trung vào một mục tiêu duy nhất: Luôn sẵn sàng khai hỏa khi bạn cần. Hoạt động ổn định, dễ bảo trì, xứng đáng là người bạn đồng hành tin cậy mỗi ngày.</t>
+  </si>
+  <si>
+    <t>Barrett M82</t>
+  </si>
+  <si>
+    <t>Khi khoảng cách không còn là giới hạn. Barrett M82 có khả năng xuyên thủng lớp giáp xe bọc thép từ khoảng cách hàng cây số. Đây là món đầu tư đắt giá dành cho những tay săn mục tiêu hạng nặng, mang lại uy lực tuyệt đối mà không cần áp sát đối phương.</t>
+  </si>
+  <si>
+    <t>MP5 SMG</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Tinh hoa của kỹ thuật Đức. MP5 nổi tiếng với độ rung cực thấp và khả năng kiểm soát hỏa lực hoàn hảo trong không gian hẹp. Thiết kế nhỏ gọn nhưng đầy uy lực, đây là món hàng "must-have" cho các phi vụ đặc biệt yêu cầu sự tốc độ và chính xác.</t>
+  </si>
+  <si>
+    <t>Colt M1911</t>
+  </si>
+  <si>
+    <t>Một miếng ghép lịch sử nằm gọn trong lòng bàn tay. Với hơn 100 năm phục vụ, M1911 vẫn giữ nguyên sức hút nhờ vẻ ngoài cơ bắp và cỡ đạn .45 ACP uy lực. Đây không chỉ là vũ khí, mà là một món đồ sưu tầm có giá trị vượt thời gian.</t>
+  </si>
+  <si>
+    <t>FN P90</t>
+  </si>
+  <si>
+    <t>Belgium</t>
+  </si>
+  <si>
+    <t>Độc đáo với băng đạn nằm ngang và thiết kế công thái học lạ mắt. P90 mang lại tốc độ bắn cực nhanh và khả năng xuyên giáp đáng kinh ngạc trong một thân hình cực kỳ nhỏ gọn. Một món hàng công nghệ cao giúp bạn nổi bật ở bất cứ đâu.</t>
+  </si>
+  <si>
+    <t>Dragunov SVD</t>
+  </si>
+  <si>
+    <t>Mẫu súng bắn tỉa huyền thoại với báng gỗ cổ điển. SVD được thiết kế để mang lại sự hỗ trợ hỏa lực tầm trung hoàn hảo cho bộ binh. Thanh mảnh nhưng chết chóc, đây là sự kết hợp giữa nét đẹp truyền thống và hiệu suất chiến đấu lạnh lùng của Nga.</t>
+  </si>
+  <si>
+    <t>Remington 870</t>
+  </si>
+  <si>
+    <t>Vũ khí tối thượng để bảo vệ tổ ấm. Với tiếng lên đạn "xoạch xoạch" đặc trưng, Remington 870 đủ sức răn đe bất kỳ kẻ đột nhập nào. Sức công phá diện rộng ở cự ly gần giúp bạn làm chủ mọi tình huống mà không cần kỹ năng nhắm bắn quá phức tạp.</t>
+  </si>
+  <si>
+    <t>1. M1 Bazooka</t>
+  </si>
+  <si>
+    <t>Mẫu thiết kế đặt nền móng cho mọi loại súng chống tăng hiện đại. Với cấu trúc ống phóng đơn giản, đây là món đồ phải có cho những người yêu thích lịch sử quân sự. Nhẹ nhàng, dễ sử dụng, nó là minh chứng cho việc sức mạnh đôi khi đến từ những thiết kế tối giản nhất.</t>
+  </si>
+  <si>
+    <t>RPG-7</t>
+  </si>
+  <si>
+    <t>Được mệnh danh là "AK-47 của dòng súng chống tăng". RPG-7 nổi tiếng nhờ giá thành rẻ và khả năng hoạt động cực kỳ tin cậy trong mọi môi trường khắc nghiệt. Chỉ cần đặt lên vai, bóp cò và xem sức mạnh của đầu đạn nổ lõm phá hủy mục tiêu một cách ngoạn mục.</t>
+  </si>
+  <si>
+    <t>FGM-148 Javelin</t>
+  </si>
+  <si>
+    <t>Mặt hàng cao cấp nhất dành cho các "đại gia" chiến trường. Với chế độ "Bắn và Quên", tên lửa tự động khóa mục tiêu và tấn công từ trên nóc—nơi yếu nhất của xe tăng. Độ chính xác tuyệt đối, công nghệ dẫn đường hồng ngoại biến mọi nỗ lực ẩn nấp của đối phương thành vô nghĩa.</t>
+  </si>
+  <si>
+    <t>Carl Gustaf M4</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>Không chỉ chống tăng, đây là một hệ thống vũ khí đa nhiệm. Carl Gustaf M4 có thể bắn được nhiều loại đạn từ nổ mạnh, xuyên giáp đến chiếu sáng. Trọng lượng siêu nhẹ nhờ vật liệu carbon hiện đại, đây là món đồ chơi công nghệ cao cho các đơn vị cơ động.</t>
+  </si>
+  <si>
+    <t>Panzerfaust 3</t>
+  </si>
+  <si>
+    <t>Tinh hoa cơ khí Đức dành cho việc đối đầu với các loại xe tăng hiện đại nhất. Với khả năng xuyên thủng giáp phản ứng nổ (ERA), Panzerfaust 3 là nỗi khiếp sợ của mọi kíp lái xe tăng. Thiết kế công thái học giúp việc ngắm bắn trở nên dễ dàng như một trò chơi điện tử.</t>
+  </si>
+  <si>
+    <t>AT4</t>
+  </si>
+  <si>
+    <t>Mặt hàng "dùng một lần rồi bỏ" cực kỳ tiện lợi. Không cần nạp đạn, không cần bảo trì rườm rà. Bạn chỉ cần rút chốt, ngắm và bắn. AT4 là lựa chọn hoàn hảo cho bộ binh cần hỏa lực mạnh tức thời mà không muốn mang vác cồng kềnh sau khi sử dụng.</t>
+  </si>
+  <si>
+    <t>M72 LAW</t>
+  </si>
+  <si>
+    <t>Nhỏ gọn đến mức kinh ngạc, có thể thu ngắn lại khi di chuyển. M72 LAW là món đồ tuyệt vời cho các nhiệm vụ đột kích nhanh. Dù nhỏ bé, nhưng nó đủ sức thổi bay các lô cốt hoặc xe bọc thép nhẹ, mang lại lợi thế bất ngờ trên chiến trường.</t>
+  </si>
+  <si>
+    <t>BGM-71 TOW</t>
+  </si>
+  <si>
+    <t>Hệ thống tên lửa dẫn đường bằng dây cực kỳ ổn định. TOW cho phép bạn điều chỉnh đường bay của tên lửa ngay cả sau khi bắn, đảm bảo mục tiêu không thể thoát khỏi tầm tay. Phù hợp cho việc thiết lập các điểm phòng thủ kiên cố từ khoảng cách an toàn.</t>
+  </si>
+  <si>
+    <t>NLAW</t>
+  </si>
+  <si>
+    <t>Chuyên gia tác chiến trong thành phố. NLAW có khả năng bắn từ không gian hẹp mà không gây nguy hiểm cho người bắn. Hệ thống dự đoán đường bay thông minh giúp tiêu diệt các mục tiêu đang di chuyển chỉ với một nút bấm. Một món hàng tinh tế và hiệu quả.</t>
+  </si>
+  <si>
+    <t>9K135 Kornet</t>
+  </si>
+  <si>
+    <t>Được thiết kế để xuyên thủng những lớp giáp dày nhất thế giới bằng công nghệ dẫn đường laser. Kornet mang lại uy lực hủy diệt ở tầm xa cực lớn. Đây là giải pháp "phá giáp" đáng tin cậy dành cho những ai tin dùng vũ khí hệ Nga.</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_01.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_10.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_09.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_08.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_07.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_06.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_05.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_04.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_03.jpg</t>
+  </si>
+  <si>
+    <t>bazooka/bazooka_02.jpg</t>
   </si>
 </sst>
 </file>
@@ -1478,7 +1940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -3811,6 +4273,1156 @@
         <v>259</v>
       </c>
     </row>
+    <row r="102" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A102" s="1">
+        <v>11</v>
+      </c>
+      <c r="B102" s="1">
+        <v>3</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="E102" s="1">
+        <v>640000</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A103" s="1">
+        <v>11</v>
+      </c>
+      <c r="B103" s="1">
+        <v>3</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="E103" s="1">
+        <v>630000</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A104" s="1">
+        <v>11</v>
+      </c>
+      <c r="B104" s="1">
+        <v>3</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="E104" s="1">
+        <v>347000</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A105" s="1">
+        <v>11</v>
+      </c>
+      <c r="B105" s="1">
+        <v>3</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E105" s="1">
+        <v>138000</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" ht="144" x14ac:dyDescent="0.3">
+      <c r="A106" s="1">
+        <v>11</v>
+      </c>
+      <c r="B106" s="1">
+        <v>3</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E106" s="1">
+        <v>1750000</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A107" s="1">
+        <v>11</v>
+      </c>
+      <c r="B107" s="1">
+        <v>3</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E107" s="1">
+        <v>360000</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A108" s="1">
+        <v>11</v>
+      </c>
+      <c r="B108" s="1">
+        <v>3</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E108" s="1">
+        <v>827500</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A109" s="1">
+        <v>11</v>
+      </c>
+      <c r="B109" s="1">
+        <v>3</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E109" s="1">
+        <v>8960000</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A110" s="1">
+        <v>11</v>
+      </c>
+      <c r="B110" s="1">
+        <v>3</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E110" s="1">
+        <v>318000</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="230.4" x14ac:dyDescent="0.3">
+      <c r="A111" s="1">
+        <v>11</v>
+      </c>
+      <c r="B111" s="1">
+        <v>3</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E111" s="1">
+        <v>827000</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A112" s="1">
+        <v>12</v>
+      </c>
+      <c r="B112" s="1">
+        <v>2</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E112" s="1">
+        <v>350000</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
+        <v>12</v>
+      </c>
+      <c r="B113" s="1">
+        <v>2</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E113" s="1">
+        <v>110000</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
+        <v>12</v>
+      </c>
+      <c r="B114" s="1">
+        <v>2</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E114" s="1">
+        <v>50000</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
+        <v>12</v>
+      </c>
+      <c r="B115" s="1">
+        <v>2</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E115" s="1">
+        <v>120000</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
+        <v>12</v>
+      </c>
+      <c r="B116" s="1">
+        <v>2</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E116" s="1">
+        <v>2100000</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>12</v>
+      </c>
+      <c r="B117" s="1">
+        <v>2</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E117" s="1">
+        <v>750000</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>12</v>
+      </c>
+      <c r="B118" s="1">
+        <v>2</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E118" s="1">
+        <v>80000</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
+        <v>12</v>
+      </c>
+      <c r="B119" s="1">
+        <v>2</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E119" s="1">
+        <v>100000</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="G119" s="1" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
+        <v>12</v>
+      </c>
+      <c r="B120" s="1">
+        <v>2</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="E120" s="1">
+        <v>100000</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
+        <v>12</v>
+      </c>
+      <c r="B121" s="1">
+        <v>2</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E121" s="1">
+        <v>111000</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>13</v>
+      </c>
+      <c r="B122" s="1">
+        <v>2</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E122" s="1">
+        <v>200000</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
+        <v>13</v>
+      </c>
+      <c r="B123" s="1">
+        <v>2</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E123" s="1">
+        <v>200000</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>13</v>
+      </c>
+      <c r="B124" s="1">
+        <v>2</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E124" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="G124" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A125" s="1">
+        <v>13</v>
+      </c>
+      <c r="B125" s="1">
+        <v>2</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E125" s="1">
+        <v>28000</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A126" s="1">
+        <v>13</v>
+      </c>
+      <c r="B126" s="1">
+        <v>2</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E126" s="1">
+        <v>25000</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="G126" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A127" s="1">
+        <v>13</v>
+      </c>
+      <c r="B127" s="1">
+        <v>2</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E127" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A128" s="1">
+        <v>13</v>
+      </c>
+      <c r="B128" s="1">
+        <v>2</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E128" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="G128" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A129" s="1">
+        <v>13</v>
+      </c>
+      <c r="B129" s="1">
+        <v>2</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E129" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="G129" s="1" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A130" s="1">
+        <v>13</v>
+      </c>
+      <c r="B130" s="1">
+        <v>2</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E130" s="1">
+        <v>70000</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="G130" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A131" s="1">
+        <v>13</v>
+      </c>
+      <c r="B131" s="1">
+        <v>2</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E131" s="1">
+        <v>31000</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="G131" s="1" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A132" s="1">
+        <v>14</v>
+      </c>
+      <c r="B132" s="1">
+        <v>1</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E132" s="1">
+        <v>1200</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="G132" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A133" s="1">
+        <v>14</v>
+      </c>
+      <c r="B133" s="1">
+        <v>1</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E133" s="1">
+        <v>1500</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="G133" s="1" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A134" s="1">
+        <v>14</v>
+      </c>
+      <c r="B134" s="1">
+        <v>1</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E134" s="1">
+        <v>2500</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="G134" s="1" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A135" s="1">
+        <v>14</v>
+      </c>
+      <c r="B135" s="1">
+        <v>1</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="E135" s="1">
+        <v>550</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="G135" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A136" s="1">
+        <v>14</v>
+      </c>
+      <c r="B136" s="1">
+        <v>1</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E136" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="G136" s="1" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A137" s="1">
+        <v>14</v>
+      </c>
+      <c r="B137" s="1">
+        <v>1</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="E137" s="1">
+        <v>3000</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="G137" s="1" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A138" s="1">
+        <v>14</v>
+      </c>
+      <c r="B138" s="1">
+        <v>1</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="D138" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E138" s="1">
+        <v>1200</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="G138" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A139" s="1">
+        <v>14</v>
+      </c>
+      <c r="B139" s="1">
+        <v>1</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="E139" s="1">
+        <v>2300</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A140" s="1">
+        <v>14</v>
+      </c>
+      <c r="B140" s="1">
+        <v>1</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E140" s="1">
+        <v>6000</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="G140" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A141" s="1">
+        <v>14</v>
+      </c>
+      <c r="B141" s="1">
+        <v>1</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="D141" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E141" s="1">
+        <v>500</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="G141" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A142" s="1">
+        <v>15</v>
+      </c>
+      <c r="B142" s="1">
+        <v>1</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E142" s="1">
+        <v>2500</v>
+      </c>
+      <c r="F142" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="G142" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A143" s="1">
+        <v>15</v>
+      </c>
+      <c r="B143" s="1">
+        <v>1</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E143" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="G143" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A144" s="1">
+        <v>15</v>
+      </c>
+      <c r="B144" s="1">
+        <v>1</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="D144" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E144" s="1">
+        <v>25000</v>
+      </c>
+      <c r="F144" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="G144" s="1" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A145" s="1">
+        <v>15</v>
+      </c>
+      <c r="B145" s="1">
+        <v>1</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="D145" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="E145" s="1">
+        <v>20000</v>
+      </c>
+      <c r="F145" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="G145" s="1" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A146" s="1">
+        <v>15</v>
+      </c>
+      <c r="B146" s="1">
+        <v>1</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="D146" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="E146" s="1">
+        <v>10000</v>
+      </c>
+      <c r="F146" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="G146" s="1" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A147" s="1">
+        <v>15</v>
+      </c>
+      <c r="B147" s="1">
+        <v>1</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="D147" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="E147" s="1">
+        <v>2500</v>
+      </c>
+      <c r="F147" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="G147" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A148" s="1">
+        <v>15</v>
+      </c>
+      <c r="B148" s="1">
+        <v>1</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="D148" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E148" s="1">
+        <v>2000</v>
+      </c>
+      <c r="F148" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="G148" s="1" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A149" s="1">
+        <v>15</v>
+      </c>
+      <c r="B149" s="1">
+        <v>1</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E149" s="1">
+        <v>50000</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="G149" s="1" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A150" s="1">
+        <v>15</v>
+      </c>
+      <c r="B150" s="1">
+        <v>1</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="D150" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E150" s="1">
+        <v>40000</v>
+      </c>
+      <c r="F150" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G150" s="1" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A151" s="1">
+        <v>15</v>
+      </c>
+      <c r="B151" s="1">
+        <v>1</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="D151" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E151" s="1">
+        <v>25000</v>
+      </c>
+      <c r="F151" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="G151" s="1" t="s">
+        <v>502</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>